<commit_message>
Update example test file CellValues
Update reference test file for example CellValues. After the style
infrastructure switch, the styles part is saved differently.
No semantic change to the styles part.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Misc/CellValues.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Misc/CellValues.xlsx
@@ -72,117 +72,73 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="0" formatCode=""/>
-    <x:numFmt numFmtId="164" formatCode="yyyy-MMM-dd"/>
-  </x:numFmts>
-  <x:fonts count="2">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="3">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF00FFFF"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="7">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="7">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-MMM-dd"/>
+  </numFmts>
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="3">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FFFF"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -486,22 +442,22 @@
   </x:cols>
   <x:sheetData>
     <x:row r="2" spans="1:7">
-      <x:c r="B2" s="1" t="s">
+      <x:c r="B2" s="6" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="C2" s="6" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="1" t="s">
+      <x:c r="D2" s="6" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="s">
+      <x:c r="E2" s="6" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="s">
+      <x:c r="F2" s="6" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G2" s="1" t="s">
+      <x:c r="G2" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -509,19 +465,19 @@
       <x:c r="B3" s="2">
         <x:v>40423</x:v>
       </x:c>
-      <x:c r="C3" s="3">
+      <x:c r="C3" s="1">
         <x:v>40423</x:v>
       </x:c>
-      <x:c r="D3" s="3">
+      <x:c r="D3" s="1">
         <x:v>40423</x:v>
       </x:c>
-      <x:c r="E3" s="3">
+      <x:c r="E3" s="1">
         <x:v>40423</x:v>
       </x:c>
-      <x:c r="F3" s="4" t="s">
+      <x:c r="F3" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G3" s="4" t="s">
+      <x:c r="G3" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -538,15 +494,15 @@
       <x:c r="E4" s="0" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F4" s="4" t="s">
+      <x:c r="F4" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G4" s="4" t="s">
+      <x:c r="G4" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
-      <x:c r="B5" s="5">
+      <x:c r="B5" s="4">
         <x:v>1234.567</x:v>
       </x:c>
       <x:c r="C5" s="0">
@@ -558,10 +514,10 @@
       <x:c r="E5" s="0">
         <x:v>1234.567</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="s">
+      <x:c r="F5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="G5" s="4" t="s">
+      <x:c r="G5" s="3" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -586,22 +542,22 @@
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
-      <x:c r="B7" s="6">
+      <x:c r="B7" s="5">
         <x:v>1.10538194444444</x:v>
       </x:c>
-      <x:c r="C7" s="6">
+      <x:c r="C7" s="5">
         <x:v>1.10538194444444</x:v>
       </x:c>
-      <x:c r="D7" s="6">
+      <x:c r="D7" s="5">
         <x:v>1.10538194444444</x:v>
       </x:c>
-      <x:c r="E7" s="6">
+      <x:c r="E7" s="5">
         <x:v>1.10538194444444</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="s">
+      <x:c r="F7" s="3" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="G7" s="4" t="s">
+      <x:c r="G7" s="3" t="s">
         <x:v>12</x:v>
       </x:c>
     </x:row>
@@ -618,10 +574,10 @@
       <x:c r="E8" s="0" t="e">
         <x:v>#DIV/0!</x:v>
       </x:c>
-      <x:c r="F8" s="4" t="s">
+      <x:c r="F8" s="3" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="G8" s="4" t="s">
+      <x:c r="G8" s="3" t="s">
         <x:v>13</x:v>
       </x:c>
     </x:row>
@@ -643,7 +599,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="4" t="s">
+      <x:c r="A1" s="3" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>

</xml_diff>